<commit_message>
Spread synthetic interventions over more lines
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014dpgFKCfBH5RfYB9JEWbof
</commit_message>
<xml_diff>
--- a/dashboard principale/data/data.xlsx
+++ b/dashboard principale/data/data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="51">
   <si>
     <t>DLigne</t>
   </si>
@@ -67,97 +67,100 @@
     <t>action faite par FSI meme avant d'entrer de saisir un eréclamation sur extranet</t>
   </si>
   <si>
-    <t>DL-002149</t>
-  </si>
-  <si>
-    <t>DL-010492</t>
-  </si>
-  <si>
-    <t>DL-002656</t>
-  </si>
-  <si>
-    <t>25.01.01.010</t>
-  </si>
-  <si>
-    <t>25.01.01.047</t>
-  </si>
-  <si>
-    <t>25.01.01.045</t>
-  </si>
-  <si>
-    <t>IM30934599</t>
-  </si>
-  <si>
-    <t>IM30934600</t>
-  </si>
-  <si>
-    <t>IM30934601</t>
+    <t>DL-010445</t>
+  </si>
+  <si>
+    <t>DL-002988</t>
+  </si>
+  <si>
+    <t>DL-005105</t>
+  </si>
+  <si>
+    <t>25.01.01.019</t>
+  </si>
+  <si>
+    <t>25.01.01.038</t>
+  </si>
+  <si>
+    <t>25.01.01.015</t>
+  </si>
+  <si>
+    <t>IM30970573</t>
+  </si>
+  <si>
+    <t>IM30970574</t>
+  </si>
+  <si>
+    <t>IM30970575</t>
   </si>
   <si>
     <t>Clôturé</t>
   </si>
   <si>
-    <t>Aucun</t>
-  </si>
-  <si>
-    <t>IPMSAN</t>
-  </si>
-  <si>
-    <t>Problème FSI</t>
+    <t>Distribution</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>NABEUL</t>
+  </si>
+  <si>
+    <t>BIZERTE</t>
   </si>
   <si>
     <t>BENAROUS</t>
   </si>
   <si>
-    <t>NABEUL</t>
-  </si>
-  <si>
-    <t>MANNOUBA</t>
-  </si>
-  <si>
-    <t>Gros ADSL postpayee</t>
-  </si>
-  <si>
     <t>Offre de Gros ADSL Hybride</t>
   </si>
   <si>
+    <t>Débit lent</t>
+  </si>
+  <si>
     <t>Déconnexion courante</t>
   </si>
   <si>
     <t>Pas de synchronisation</t>
   </si>
   <si>
-    <t>10 mbps</t>
+    <t>12 mbps</t>
   </si>
   <si>
     <t>20 mbps</t>
   </si>
   <si>
+    <t>4 mbps</t>
+  </si>
+  <si>
     <t>Hexabyte</t>
   </si>
   <si>
-    <t>Fixation Coffret</t>
-  </si>
-  <si>
-    <t>Client absent</t>
+    <t>Relève Isolement</t>
+  </si>
+  <si>
+    <t>Rien à signaler</t>
   </si>
   <si>
     <t>Remplacement Jarretière</t>
   </si>
   <si>
+    <t>Ret</t>
+  </si>
+  <si>
     <t>Isolement</t>
   </si>
   <si>
-    <t>Coffret fixé</t>
-  </si>
-  <si>
-    <t>0 03:34:29</t>
-  </si>
-  <si>
-    <t>3 09:32:32</t>
-  </si>
-  <si>
-    <t>0 08:37:22</t>
+    <t>3 05:44:59</t>
+  </si>
+  <si>
+    <t>0 18:24:20</t>
+  </si>
+  <si>
+    <t>0 04:52:19</t>
+  </si>
+  <si>
+    <t>état modem : Connecté Perte de synchro : Oui Déconnexion sans filtre : Oui Message FSI : Connexion établie au moins une fois.</t>
   </si>
   <si>
     <t>Débit mesuré inférieur au débit souscrit, test effectué sans filtre, merci de vérifier la ligne.</t>
@@ -563,10 +566,10 @@
         <v>20</v>
       </c>
       <c r="C2" s="1">
-        <v>45658.27138850861</v>
+        <v>45658.27462801851</v>
       </c>
       <c r="D2" s="1">
-        <v>45658.2716973416</v>
+        <v>45658.27492092875</v>
       </c>
       <c r="E2" t="s">
         <v>23</v>
@@ -575,22 +578,22 @@
         <v>26</v>
       </c>
       <c r="G2" s="1">
-        <v>45658.42064448038</v>
+        <v>45661.51450314173</v>
       </c>
       <c r="H2" t="s">
         <v>27</v>
       </c>
       <c r="I2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K2" t="s">
         <v>33</v>
       </c>
-      <c r="K2" t="s">
-        <v>35</v>
-      </c>
       <c r="L2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M2" t="s">
         <v>39</v>
@@ -616,10 +619,10 @@
         <v>21</v>
       </c>
       <c r="C3" s="1">
-        <v>45658.28314136943</v>
+        <v>45658.29267377396</v>
       </c>
       <c r="D3" s="1">
-        <v>45658.28338110743</v>
+        <v>45658.29308080647</v>
       </c>
       <c r="E3" t="s">
         <v>24</v>
@@ -628,31 +631,28 @@
         <v>26</v>
       </c>
       <c r="G3" s="1">
-        <v>45661.6809836985</v>
+        <v>45659.05998185236</v>
       </c>
       <c r="H3" t="s">
         <v>28</v>
       </c>
       <c r="I3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" t="s">
         <v>34</v>
       </c>
-      <c r="K3" t="s">
-        <v>35</v>
-      </c>
       <c r="L3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M3" t="s">
         <v>39</v>
       </c>
       <c r="N3" t="s">
         <v>41</v>
-      </c>
-      <c r="O3" t="s">
-        <v>43</v>
       </c>
       <c r="P3" t="s">
         <v>46</v>
@@ -669,10 +669,10 @@
         <v>22</v>
       </c>
       <c r="C4" s="1">
-        <v>45658.30140287846</v>
+        <v>45658.32514736393</v>
       </c>
       <c r="D4" s="1">
-        <v>45658.30143344384</v>
+        <v>45658.32522136846</v>
       </c>
       <c r="E4" t="s">
         <v>25</v>
@@ -681,19 +681,19 @@
         <v>26</v>
       </c>
       <c r="G4" s="1">
-        <v>45658.66071936092</v>
+        <v>45658.52821922087</v>
       </c>
       <c r="H4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" t="s">
         <v>32</v>
       </c>
-      <c r="J4" t="s">
-        <v>33</v>
-      </c>
       <c r="K4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L4" t="s">
         <v>38</v>
@@ -711,7 +711,7 @@
         <v>47</v>
       </c>
       <c r="Q4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>